<commit_message>
Drop em dashes and the What changed section from the RACI deliverables
Alvin's instruction: no em dashes, and the team-facing page does not need a
version-history block. Version history stays in deliverables/README.md.

- build_html.py: removed the CHANGES constant, its markup and its CSS; replaced
  every em and en dash in the template, including the details open marker, which
  now renders a true minus sign
- build_raci.py: the Analysis roster labels use a colon instead of a dash
- raci_rows.py: one row note reworded
- Swept deliverables/README.md, references/external-partners.md and
  connections.md, repunctuating rather than substituting commas blindly
- Recorded the rule under House style in deliverables/README.md so a future
  rebuild does not reintroduce either

Regenerated all three deliverables. verify.py passes all seven checks: 102 rows,
one A and one R each, 245 citations resolve, no partner holds accountability, no
open seat holds a letter, nine role-maps in sync.
</commit_message>
<xml_diff>
--- a/deliverables/AC-Brands-RACI.xlsx
+++ b/deliverables/AC-Brands-RACI.xlsx
@@ -2665,7 +2665,7 @@
       </c>
       <c r="W32" s="6" t="inlineStr">
         <is>
-          <t>The strictest gate in the suite: explicit approval at every step, §4.A through §4.F each a separate gate. Operator decides severity, team and whether external reporting is needed. A and R both AB. Stays with Alvin as Reg Lead — legal and agency exposure. Nicole consults. Pedrero Regulatory holds the binding external review; consult-only internally, with no Asana access and no internal authority, so the Reg Lead gate stays in-house.</t>
+          <t>The strictest gate in the suite: explicit approval at every step, §4.A through §4.F each a separate gate. Operator decides severity, team and whether external reporting is needed. A and R both AB. Stays with Alvin as Reg Lead, given the legal and agency exposure. Nicole consults. Pedrero Regulatory holds the binding external review; consult-only internally, with no Asana access and no internal authority, so the Reg Lead gate stays in-house.</t>
         </is>
       </c>
     </row>
@@ -7923,7 +7923,7 @@
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>AC — Owner / Founder (Ayesha Curry)</t>
+          <t>AC: Owner / Founder (Ayesha Curry)</t>
         </is>
       </c>
       <c r="B6" s="15">
@@ -7956,7 +7956,7 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>DI — President (Danielle Iturbe)</t>
+          <t>DI: President (Danielle Iturbe)</t>
         </is>
       </c>
       <c r="B7" s="15">
@@ -7989,7 +7989,7 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>AB — VP of Operations (Alvin Belt)</t>
+          <t>AB: VP of Operations (Alvin Belt)</t>
         </is>
       </c>
       <c r="B8" s="15">
@@ -8022,7 +8022,7 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>NI — Sr. Director, Consumer Strategy &amp; Operations (Nicole Iturbe)</t>
+          <t>NI: Sr. Director, Consumer Strategy &amp; Operations (Nicole Iturbe)</t>
         </is>
       </c>
       <c r="B9" s="15">
@@ -8055,7 +8055,7 @@
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>OPS — Operations Specialist (Open seat)</t>
+          <t>OPS: Operations Specialist (Open seat)</t>
         </is>
       </c>
       <c r="B10" s="15">
@@ -8088,7 +8088,7 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>PDS — Product Development Specialist (Open seat)</t>
+          <t>PDS: Product Development Specialist (Open seat)</t>
         </is>
       </c>
       <c r="B11" s="15">
@@ -8121,7 +8121,7 @@
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>SS — Marketing Manager (Soraya Salgadoe)</t>
+          <t>SS: Marketing Manager (Soraya Salgadoe)</t>
         </is>
       </c>
       <c r="B12" s="15">
@@ -8154,7 +8154,7 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>KL — Social Media Coordinator (Kate Le)</t>
+          <t>KL: Social Media Coordinator (Kate Le)</t>
         </is>
       </c>
       <c r="B13" s="15">
@@ -8187,7 +8187,7 @@
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>EH — Creative Director (Erin Hover)</t>
+          <t>EH: Creative Director (Erin Hover)</t>
         </is>
       </c>
       <c r="B14" s="15">
@@ -8220,7 +8220,7 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>IT — Creative / Design Coordinator (Ivy Tan)</t>
+          <t>IT: Creative / Design Coordinator (Ivy Tan)</t>
         </is>
       </c>
       <c r="B15" s="15">
@@ -8253,7 +8253,7 @@
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>JH — Packaging Engineer (Jan Haeck)</t>
+          <t>JH: Packaging Engineer (Jan Haeck)</t>
         </is>
       </c>
       <c r="B16" s="15">
@@ -8286,7 +8286,7 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>PC — PD / R&amp;D contractor, Milinyc (Perrine Calvet)</t>
+          <t>PC: PD / R&amp;D contractor, Milinyc (Perrine Calvet)</t>
         </is>
       </c>
       <c r="B17" s="15">
@@ -8319,7 +8319,7 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>PR — External regulatory partner (Pedrero Regulatory)</t>
+          <t>PR: External regulatory partner (Pedrero Regulatory)</t>
         </is>
       </c>
       <c r="B18" s="15">
@@ -8352,7 +8352,7 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>IF — Outsourced finance (Dan Bender) (Ironclad Finance)</t>
+          <t>IF: Outsourced finance (Dan Bender) (Ironclad Finance)</t>
         </is>
       </c>
       <c r="B19" s="15">
@@ -8385,7 +8385,7 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>CH — PEO and co-employer (Calm HR)</t>
+          <t>CH: PEO and co-employer (Calm HR)</t>
         </is>
       </c>
       <c r="B20" s="15">
@@ -8418,7 +8418,7 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>WI — Digital marketing agency (WITHIN)</t>
+          <t>WI: Digital marketing agency (WITHIN)</t>
         </is>
       </c>
       <c r="B21" s="15">
@@ -8451,7 +8451,7 @@
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>TK — Web development (Teknologics)</t>
+          <t>TK: Web development (Teknologics)</t>
         </is>
       </c>
       <c r="B22" s="15">
@@ -8484,7 +8484,7 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>CI — Managed IT service provider (Coastal Interactive)</t>
+          <t>CI: Managed IT service provider (Coastal Interactive)</t>
         </is>
       </c>
       <c r="B23" s="15">

</xml_diff>

<commit_message>
RACI deliverables: no em dashes, no What changed section (#25)
Editorial pass. Em dashes and en dashes removed from the HTML page, the
summary, the xlsx, the build scripts, deliverables/README.md,
references/external-partners.md and connections.md, repunctuated line by
line. The team page's What changed section is gone; version history stays
in deliverables/README.md. Both rules recorded under House style.

No row data, ownership or counts changed. verify.py passes all seven checks.
</commit_message>
<xml_diff>
--- a/deliverables/AC-Brands-RACI.xlsx
+++ b/deliverables/AC-Brands-RACI.xlsx
@@ -2665,7 +2665,7 @@
       </c>
       <c r="W32" s="6" t="inlineStr">
         <is>
-          <t>The strictest gate in the suite: explicit approval at every step, §4.A through §4.F each a separate gate. Operator decides severity, team and whether external reporting is needed. A and R both AB. Stays with Alvin as Reg Lead — legal and agency exposure. Nicole consults. Pedrero Regulatory holds the binding external review; consult-only internally, with no Asana access and no internal authority, so the Reg Lead gate stays in-house.</t>
+          <t>The strictest gate in the suite: explicit approval at every step, §4.A through §4.F each a separate gate. Operator decides severity, team and whether external reporting is needed. A and R both AB. Stays with Alvin as Reg Lead, given the legal and agency exposure. Nicole consults. Pedrero Regulatory holds the binding external review; consult-only internally, with no Asana access and no internal authority, so the Reg Lead gate stays in-house.</t>
         </is>
       </c>
     </row>
@@ -7923,7 +7923,7 @@
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>AC — Owner / Founder (Ayesha Curry)</t>
+          <t>AC: Owner / Founder (Ayesha Curry)</t>
         </is>
       </c>
       <c r="B6" s="15">
@@ -7956,7 +7956,7 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>DI — President (Danielle Iturbe)</t>
+          <t>DI: President (Danielle Iturbe)</t>
         </is>
       </c>
       <c r="B7" s="15">
@@ -7989,7 +7989,7 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>AB — VP of Operations (Alvin Belt)</t>
+          <t>AB: VP of Operations (Alvin Belt)</t>
         </is>
       </c>
       <c r="B8" s="15">
@@ -8022,7 +8022,7 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>NI — Sr. Director, Consumer Strategy &amp; Operations (Nicole Iturbe)</t>
+          <t>NI: Sr. Director, Consumer Strategy &amp; Operations (Nicole Iturbe)</t>
         </is>
       </c>
       <c r="B9" s="15">
@@ -8055,7 +8055,7 @@
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>OPS — Operations Specialist (Open seat)</t>
+          <t>OPS: Operations Specialist (Open seat)</t>
         </is>
       </c>
       <c r="B10" s="15">
@@ -8088,7 +8088,7 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>PDS — Product Development Specialist (Open seat)</t>
+          <t>PDS: Product Development Specialist (Open seat)</t>
         </is>
       </c>
       <c r="B11" s="15">
@@ -8121,7 +8121,7 @@
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>SS — Marketing Manager (Soraya Salgadoe)</t>
+          <t>SS: Marketing Manager (Soraya Salgadoe)</t>
         </is>
       </c>
       <c r="B12" s="15">
@@ -8154,7 +8154,7 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>KL — Social Media Coordinator (Kate Le)</t>
+          <t>KL: Social Media Coordinator (Kate Le)</t>
         </is>
       </c>
       <c r="B13" s="15">
@@ -8187,7 +8187,7 @@
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>EH — Creative Director (Erin Hover)</t>
+          <t>EH: Creative Director (Erin Hover)</t>
         </is>
       </c>
       <c r="B14" s="15">
@@ -8220,7 +8220,7 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>IT — Creative / Design Coordinator (Ivy Tan)</t>
+          <t>IT: Creative / Design Coordinator (Ivy Tan)</t>
         </is>
       </c>
       <c r="B15" s="15">
@@ -8253,7 +8253,7 @@
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>JH — Packaging Engineer (Jan Haeck)</t>
+          <t>JH: Packaging Engineer (Jan Haeck)</t>
         </is>
       </c>
       <c r="B16" s="15">
@@ -8286,7 +8286,7 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>PC — PD / R&amp;D contractor, Milinyc (Perrine Calvet)</t>
+          <t>PC: PD / R&amp;D contractor, Milinyc (Perrine Calvet)</t>
         </is>
       </c>
       <c r="B17" s="15">
@@ -8319,7 +8319,7 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>PR — External regulatory partner (Pedrero Regulatory)</t>
+          <t>PR: External regulatory partner (Pedrero Regulatory)</t>
         </is>
       </c>
       <c r="B18" s="15">
@@ -8352,7 +8352,7 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>IF — Outsourced finance (Dan Bender) (Ironclad Finance)</t>
+          <t>IF: Outsourced finance (Dan Bender) (Ironclad Finance)</t>
         </is>
       </c>
       <c r="B19" s="15">
@@ -8385,7 +8385,7 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>CH — PEO and co-employer (Calm HR)</t>
+          <t>CH: PEO and co-employer (Calm HR)</t>
         </is>
       </c>
       <c r="B20" s="15">
@@ -8418,7 +8418,7 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>WI — Digital marketing agency (WITHIN)</t>
+          <t>WI: Digital marketing agency (WITHIN)</t>
         </is>
       </c>
       <c r="B21" s="15">
@@ -8451,7 +8451,7 @@
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>TK — Web development (Teknologics)</t>
+          <t>TK: Web development (Teknologics)</t>
         </is>
       </c>
       <c r="B22" s="15">
@@ -8484,7 +8484,7 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>CI — Managed IT service provider (Coastal Interactive)</t>
+          <t>CI: Managed IT service provider (Coastal Interactive)</t>
         </is>
       </c>
       <c r="B23" s="15">

</xml_diff>